<commit_message>
The Cross Map: comparison rebuilt as five-platform on every table
- Every time-series table now carries all five machines (Athene, GA,
  BNT, Aspida, Kuvare) with per-platform color rows; dotted cells are
  disclosure facts (BNT quarterly began 1Q25; Aspida/Kuvare have no
  quarterly cadence; derived rates flagged).
- New measurable: BNT annuity spread derived from printed segment
  dollars - 1.90% (4Q24) -> 1.76% (1Q26), cost of funds up every
  quarter; Aspida/KLR derived earned rates; KLR negative equity visible
  in the equity row; Aspida deposit-type 0 -> $819M.
- Quality table adds the AEL position-drill control rows (PL trend,
  below-IG, 4.0y age); capital table has all four public ECR pivots +
  Brookfield no-FCR boundary + five lead-carrier capital rows.
- BNT workbook: annuity ruler rows were dollars mis-formatted as %;
  fixed + derived-rate formulas added (93 checks, 0 fail).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dossiers/brookfield/bnt-quarterly-engine.xlsx
+++ b/dossiers/brookfield/bnt-quarterly-engine.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -82,8 +81,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1793,7 +1792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -2304,855 +2303,979 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>② THE ANNUITY RULER — rates (printed, %)</t>
+          <t>② THE ANNUITY RULER — segment dollars (printed) and derived annualized rates</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Annuity net investment income (rate)</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
+          <t>Annuity net investment income</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
         <v>1220</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C24" s="3" t="n">
         <v>1321</v>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="D24" s="3" t="n">
         <v>1345</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E24" s="3" t="n">
         <v>1371</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="3" t="n">
         <v>1416</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="G24" s="3" t="n">
         <v>1487</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Annuity cost of funds (rate)</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
+          <t>Annuity cost of funds</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
         <v>-804</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C25" s="3" t="n">
         <v>-899</v>
       </c>
-      <c r="D25" s="5" t="n">
+      <c r="D25" s="3" t="n">
         <v>-935</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="E25" s="3" t="n">
         <v>-972</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="3" t="n">
         <v>-984</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="G25" s="3" t="n">
         <v>-1031</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ANNUITY NET INVESTMENT SPREAD</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
+          <t>ANNUITY NET INVESTMENT SPREAD (printed)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
         <v>416</v>
       </c>
-      <c r="C26" s="5" t="n">
+      <c r="C26" s="3" t="n">
         <v>422</v>
       </c>
-      <c r="D26" s="5" t="n">
+      <c r="D26" s="3" t="n">
         <v>410</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="E26" s="3" t="n">
         <v>399</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="3" t="n">
         <v>432</v>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="G26" s="3" t="n">
         <v>456</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>CHECK: NII + cost of funds = net spread</t>
+        </is>
+      </c>
+      <c r="B27" s="4">
+        <f>IF(OR(B24+B25="",B26=""),"n/a",IF(ABS(B24+B25-B26)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="C27" s="4">
+        <f>IF(OR(C24+C25="",C26=""),"n/a",IF(ABS(C24+C25-C26)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="D27" s="4">
+        <f>IF(OR(D24+D25="",D26=""),"n/a",IF(ABS(D24+D25-D26)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="E27" s="4">
+        <f>IF(OR(E24+E25="",E26=""),"n/a",IF(ABS(E24+E25-E26)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="F27" s="4">
+        <f>IF(OR(F24+F25="",F26=""),"n/a",IF(ABS(F24+F25-F26)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="G27" s="4">
+        <f>IF(OR(G24+G25="",G26=""),"n/a",IF(ABS(G24+G25-G26)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Annuity average invested assets</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B28" s="3" t="n">
         <v>87507</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C28" s="3" t="n">
         <v>91266</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D28" s="3" t="n">
         <v>93479</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E28" s="3" t="n">
         <v>96527</v>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F28" s="3" t="n">
         <v>100708</v>
       </c>
-      <c r="G27" s="3" t="n">
+      <c r="G28" s="3" t="n">
         <v>103465</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Earned rate (derived, ×4 / avg invested assets)</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>IF(B28=0,"",B24*4/B28)</f>
+        <v/>
+      </c>
+      <c r="C29" s="6">
+        <f>IF(C28=0,"",C24*4/C28)</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>IF(D28=0,"",D24*4/D28)</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>IF(E28=0,"",E24*4/E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="6">
+        <f>IF(F28=0,"",F24*4/F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="6">
+        <f>IF(G28=0,"",G24*4/G28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Cost of funds rate (derived)</t>
+        </is>
+      </c>
+      <c r="B30" s="6">
+        <f>IF(B28=0,"",B25*4/B28)</f>
+        <v/>
+      </c>
+      <c r="C30" s="6">
+        <f>IF(C28=0,"",C25*4/C28)</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>IF(D28=0,"",D25*4/D28)</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>IF(E28=0,"",E25*4/E28)</f>
+        <v/>
+      </c>
+      <c r="F30" s="6">
+        <f>IF(F28=0,"",F25*4/F28)</f>
+        <v/>
+      </c>
+      <c r="G30" s="6">
+        <f>IF(G28=0,"",G25*4/G28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>NET INVESTMENT SPREAD rate (derived)</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>IF(B28=0,"",B26*4/B28)</f>
+        <v/>
+      </c>
+      <c r="C31" s="6">
+        <f>IF(C28=0,"",C26*4/C28)</f>
+        <v/>
+      </c>
+      <c r="D31" s="6">
+        <f>IF(D28=0,"",D26*4/D28)</f>
+        <v/>
+      </c>
+      <c r="E31" s="6">
+        <f>IF(E28=0,"",E26*4/E28)</f>
+        <v/>
+      </c>
+      <c r="F31" s="6">
+        <f>IF(F28=0,"",F26*4/F28)</f>
+        <v/>
+      </c>
+      <c r="G31" s="6">
+        <f>IF(G28=0,"",G26*4/G28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>③ FLOWS — sales, outflows, net flows</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">    Retail sales — fixed index</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B34" s="3" t="n">
         <v>1797</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C34" s="3" t="n">
         <v>1835</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D34" s="3" t="n">
         <v>2513</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E34" s="3" t="n">
         <v>2529</v>
       </c>
-      <c r="F30" s="3" t="n">
+      <c r="F34" s="3" t="n">
         <v>2155</v>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="G34" s="3" t="n">
         <v>1691</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Retail sales — fixed rate</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="n">
-        <v>918</v>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>1049</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>1031</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>2128</v>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>2028</v>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>1385</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Retail sales — variable/other</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>80</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>101</v>
-      </c>
-      <c r="F32" s="3" t="n">
-        <v>166</v>
-      </c>
-      <c r="G32" s="3" t="n">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Total retail sales (printed)</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="n">
-        <v>2731</v>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>2930</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>3624</v>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>4758</v>
-      </c>
-      <c r="F33" s="3" t="n">
-        <v>4349</v>
-      </c>
-      <c r="G33" s="3" t="n">
-        <v>3252</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>CHECK: retail foots</t>
-        </is>
-      </c>
-      <c r="B34" s="4">
-        <f>IF(OR(B30+B31+B32="",B33=""),"n/a",IF(ABS(B30+B31+B32-B33)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="C34" s="4">
-        <f>IF(OR(C30+C31+C32="",C33=""),"n/a",IF(ABS(C30+C31+C32-C33)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="D34" s="4">
-        <f>IF(OR(D30+D31+D32="",D33=""),"n/a",IF(ABS(D30+D31+D32-D33)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="E34" s="4">
-        <f>IF(OR(E30+E31+E32="",E33=""),"n/a",IF(ABS(E30+E31+E32-E33)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="F34" s="4">
-        <f>IF(OR(F30+F31+F32="",F33=""),"n/a",IF(ABS(F30+F31+F32-F33)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="G34" s="4">
-        <f>IF(OR(G30+G31+G32="",G33=""),"n/a",IF(ABS(G30+G31+G32-G33)&lt;=2,"OK","FAIL"))</f>
-        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Institutional — PRT</t>
+          <t xml:space="preserve">    Retail sales — fixed rate</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>3241</v>
+        <v>918</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>408</v>
+        <v>1049</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>311</v>
+        <v>1031</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>280</v>
+        <v>2128</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>880</v>
+        <v>2028</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>90</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Institutional — funding agreements</t>
+          <t xml:space="preserve">    Retail sales — variable/other</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>500</v>
+        <v>46</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>400</v>
+        <v>80</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1389</v>
+        <v>166</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>500</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Total institutional sales (printed)</t>
+          <t>Total retail sales (printed)</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>3241</v>
+        <v>2731</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>908</v>
+        <v>2930</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>711</v>
+        <v>3624</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>280</v>
+        <v>4758</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>2269</v>
+        <v>4349</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>590</v>
+        <v>3252</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>CHECK: institutional foots</t>
+          <t>CHECK: retail foots</t>
         </is>
       </c>
       <c r="B38" s="4">
-        <f>IF(OR(B35+B36="",B37=""),"n/a",IF(ABS(B35+B36-B37)&lt;=2,"OK","FAIL"))</f>
+        <f>IF(OR(B34+B35+B36="",B37=""),"n/a",IF(ABS(B34+B35+B36-B37)&lt;=2,"OK","FAIL"))</f>
         <v/>
       </c>
       <c r="C38" s="4">
-        <f>IF(OR(C35+C36="",C37=""),"n/a",IF(ABS(C35+C36-C37)&lt;=2,"OK","FAIL"))</f>
+        <f>IF(OR(C34+C35+C36="",C37=""),"n/a",IF(ABS(C34+C35+C36-C37)&lt;=2,"OK","FAIL"))</f>
         <v/>
       </c>
       <c r="D38" s="4">
-        <f>IF(OR(D35+D36="",D37=""),"n/a",IF(ABS(D35+D36-D37)&lt;=2,"OK","FAIL"))</f>
+        <f>IF(OR(D34+D35+D36="",D37=""),"n/a",IF(ABS(D34+D35+D36-D37)&lt;=2,"OK","FAIL"))</f>
         <v/>
       </c>
       <c r="E38" s="4">
-        <f>IF(OR(E35+E36="",E37=""),"n/a",IF(ABS(E35+E36-E37)&lt;=2,"OK","FAIL"))</f>
+        <f>IF(OR(E34+E35+E36="",E37=""),"n/a",IF(ABS(E34+E35+E36-E37)&lt;=2,"OK","FAIL"))</f>
         <v/>
       </c>
       <c r="F38" s="4">
-        <f>IF(OR(F35+F36="",F37=""),"n/a",IF(ABS(F35+F36-F37)&lt;=2,"OK","FAIL"))</f>
+        <f>IF(OR(F34+F35+F36="",F37=""),"n/a",IF(ABS(F34+F35+F36-F37)&lt;=2,"OK","FAIL"))</f>
         <v/>
       </c>
       <c r="G38" s="4">
-        <f>IF(OR(G35+G36="",G37=""),"n/a",IF(ABS(G35+G36-G37)&lt;=2,"OK","FAIL"))</f>
+        <f>IF(OR(G34+G35+G36="",G37=""),"n/a",IF(ABS(G34+G35+G36-G37)&lt;=2,"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>TOTAL GROSS ANNUITY SALES (printed)</t>
+          <t xml:space="preserve">    Institutional — PRT</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>5972</v>
+        <v>3241</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>3838</v>
+        <v>408</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>4335</v>
+        <v>311</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>5038</v>
+        <v>280</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>6618</v>
+        <v>880</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>3842</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>CHECK: retail + institutional = gross sales</t>
-        </is>
-      </c>
-      <c r="B40" s="4">
-        <f>IF(OR(B33+B37="",B39=""),"n/a",IF(ABS(B33+B37-B39)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="C40" s="4">
-        <f>IF(OR(C33+C37="",C39=""),"n/a",IF(ABS(C33+C37-C39)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="D40" s="4">
-        <f>IF(OR(D33+D37="",D39=""),"n/a",IF(ABS(D33+D37-D39)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="E40" s="4">
-        <f>IF(OR(E33+E37="",E39=""),"n/a",IF(ABS(E33+E37-E39)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="F40" s="4">
-        <f>IF(OR(F33+F37="",F39=""),"n/a",IF(ABS(F33+F37-F39)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="G40" s="4">
-        <f>IF(OR(G33+G37="",G39=""),"n/a",IF(ABS(G33+G37-G39)&lt;=2,"OK","FAIL"))</f>
-        <v/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Institutional — funding agreements</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>1389</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">      retail outflows</t>
+          <t>Total institutional sales (printed)</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>-2246</v>
+        <v>3241</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>-2158</v>
+        <v>908</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-2475</v>
+        <v>711</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-2816</v>
+        <v>280</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-2763</v>
+        <v>2269</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>-2730</v>
+        <v>590</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      institutional outflows</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>-150</v>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>-142</v>
-      </c>
-      <c r="D42" s="3" t="n">
-        <v>-180</v>
-      </c>
-      <c r="E42" s="3" t="n">
-        <v>-201</v>
-      </c>
-      <c r="F42" s="3" t="n">
-        <v>-221</v>
-      </c>
-      <c r="G42" s="3" t="n">
-        <v>-225</v>
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>CHECK: institutional foots</t>
+        </is>
+      </c>
+      <c r="B42" s="4">
+        <f>IF(OR(B39+B40="",B41=""),"n/a",IF(ABS(B39+B40-B41)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="C42" s="4">
+        <f>IF(OR(C39+C40="",C41=""),"n/a",IF(ABS(C39+C40-C41)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="D42" s="4">
+        <f>IF(OR(D39+D40="",D41=""),"n/a",IF(ABS(D39+D40-D41)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="E42" s="4">
+        <f>IF(OR(E39+E40="",E41=""),"n/a",IF(ABS(E39+E40-E41)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="F42" s="4">
+        <f>IF(OR(F39+F40="",F41=""),"n/a",IF(ABS(F39+F40-F41)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="G42" s="4">
+        <f>IF(OR(G39+G40="",G41=""),"n/a",IF(ABS(G39+G40-G41)&lt;=2,"OK","FAIL"))</f>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Total net annuity sales (printed)</t>
+          <t>TOTAL GROSS ANNUITY SALES (printed)</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>5969</v>
+        <v>5972</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>3831</v>
+        <v>3838</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>4326</v>
+        <v>4335</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>5024</v>
+        <v>5038</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>6604</v>
+        <v>6618</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>3840</v>
+        <v>3842</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL NET FLOWS (printed)</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="n">
-        <v>3573</v>
-      </c>
-      <c r="C44" s="3" t="n">
-        <v>1531</v>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>1671</v>
-      </c>
-      <c r="E44" s="3" t="n">
-        <v>2007</v>
-      </c>
-      <c r="F44" s="3" t="n">
-        <v>3620</v>
-      </c>
-      <c r="G44" s="3" t="n">
-        <v>885</v>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>CHECK: retail + institutional = gross sales</t>
+        </is>
+      </c>
+      <c r="B44" s="4">
+        <f>IF(OR(B37+B41="",B43=""),"n/a",IF(ABS(B37+B41-B43)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="C44" s="4">
+        <f>IF(OR(C37+C41="",C43=""),"n/a",IF(ABS(C37+C41-C43)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="D44" s="4">
+        <f>IF(OR(D37+D41="",D43=""),"n/a",IF(ABS(D37+D41-D43)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="E44" s="4">
+        <f>IF(OR(E37+E41="",E43=""),"n/a",IF(ABS(E37+E41-E43)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="F44" s="4">
+        <f>IF(OR(F37+F41="",F43=""),"n/a",IF(ABS(F37+F41-F43)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="G44" s="4">
+        <f>IF(OR(G37+G41="",G43=""),"n/a",IF(ABS(G37+G41-G43)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      retail outflows</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>-2246</v>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>-2158</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>-2475</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>-2816</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>-2763</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>-2730</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>④ INCOME ROWS (GAAP basis)</t>
-        </is>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      institutional outflows</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>-150</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>-142</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>-180</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>-201</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>-221</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>-225</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Net premiums and other policy revenue</t>
+          <t>Total net annuity sales (printed)</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>4307</v>
+        <v>5969</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>1301</v>
+        <v>3831</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>1229</v>
+        <v>4326</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>1002</v>
+        <v>5024</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>1745</v>
+        <v>6604</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>872</v>
+        <v>3840</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Net investment income incl funds withheld</t>
+          <t>TOTAL NET FLOWS (printed)</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>1325</v>
+        <v>3573</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>1429</v>
+        <v>1531</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>1486</v>
+        <v>1671</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>1493</v>
+        <v>2007</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>1484</v>
+        <v>3620</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>1471</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Net investment gains (losses) incl funds withheld</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="n">
-        <v>115</v>
-      </c>
-      <c r="C49" s="3" t="n">
-        <v>-112</v>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>322</v>
-      </c>
-      <c r="E49" s="3" t="n">
-        <v>431</v>
-      </c>
-      <c r="F49" s="3" t="n">
-        <v>-175</v>
-      </c>
-      <c r="G49" s="3" t="n">
-        <v>-687</v>
+        <v>885</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>④ INCOME ROWS (GAAP basis)</t>
+        </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="inlineStr">
-        <is>
-          <t>⑤ STOCKS</t>
-        </is>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Net premiums and other policy revenue</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>4307</v>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>1301</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>1229</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>1002</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>1745</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>872</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Total assets</t>
+          <t>Net investment income incl funds withheld</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>139953</v>
+        <v>1325</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>141612</v>
+        <v>1429</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>148893</v>
+        <v>1486</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>152821</v>
+        <v>1493</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>157181</v>
+        <v>1484</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>156059</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">      total insurance assets</t>
+          <t>Net investment gains (losses) incl funds withheld</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>129698</v>
+        <v>115</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>131385</v>
+        <v>-112</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>134726</v>
+        <v>322</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>138520</v>
+        <v>431</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>143427</v>
+        <v>-175</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>143525</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Total liabilities</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="n">
-        <v>126877</v>
-      </c>
-      <c r="C54" s="3" t="n">
-        <v>128602</v>
-      </c>
-      <c r="D54" s="3" t="n">
-        <v>133054</v>
-      </c>
-      <c r="E54" s="3" t="n">
-        <v>135906</v>
-      </c>
-      <c r="F54" s="3" t="n">
-        <v>139264</v>
-      </c>
-      <c r="G54" s="3" t="n">
-        <v>139168</v>
+        <v>-687</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      total insurance liabilities</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n">
-        <v>115218</v>
-      </c>
-      <c r="C55" s="3" t="n">
-        <v>117265</v>
-      </c>
-      <c r="D55" s="3" t="n">
-        <v>120193</v>
-      </c>
-      <c r="E55" s="3" t="n">
-        <v>122872</v>
-      </c>
-      <c r="F55" s="3" t="n">
-        <v>126902</v>
-      </c>
-      <c r="G55" s="3" t="n">
-        <v>127336</v>
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>⑤ STOCKS</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">      total gross reserves</t>
+          <t>Total assets</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>109983</v>
-      </c>
-      <c r="C56" s="3" t="n"/>
-      <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="n"/>
+        <v>139953</v>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>141612</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>148893</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>152821</v>
+      </c>
       <c r="F56" s="3" t="n">
-        <v>122473</v>
+        <v>157181</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>122911</v>
+        <v>156059</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">      total net reserves</t>
+          <t xml:space="preserve">      total insurance assets</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>97894</v>
-      </c>
-      <c r="C57" s="3" t="n"/>
-      <c r="D57" s="3" t="n"/>
-      <c r="E57" s="3" t="n"/>
+        <v>129698</v>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>131385</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>134726</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>138520</v>
+      </c>
       <c r="F57" s="3" t="n">
-        <v>110321</v>
+        <v>143427</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>110974</v>
+        <v>143525</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Total equity</t>
+          <t>Total liabilities</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>13076</v>
+        <v>126877</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>13010</v>
+        <v>128602</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>15839</v>
+        <v>133054</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>16915</v>
+        <v>135906</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>17917</v>
+        <v>139264</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>16891</v>
+        <v>139168</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>CHECK: A = L + E</t>
-        </is>
-      </c>
-      <c r="B59" s="4">
-        <f>IF(OR(B54+B58="",B52=""),"n/a",IF(ABS(B54+B58-B52)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="C59" s="4">
-        <f>IF(OR(C54+C58="",C52=""),"n/a",IF(ABS(C54+C58-C52)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="D59" s="4">
-        <f>IF(OR(D54+D58="",D52=""),"n/a",IF(ABS(D54+D58-D52)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="E59" s="4">
-        <f>IF(OR(E54+E58="",E52=""),"n/a",IF(ABS(E54+E58-E52)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="F59" s="4">
-        <f>IF(OR(F54+F58="",F52=""),"n/a",IF(ABS(F54+F58-F52)&lt;=2,"OK","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="G59" s="4">
-        <f>IF(OR(G54+G58="",G52=""),"n/a",IF(ABS(G54+G58-G52)&lt;=2,"OK","FAIL"))</f>
-        <v/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      total insurance liabilities</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n">
+        <v>115218</v>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>117265</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>120193</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>122872</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>126902</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>127336</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Adjusted equity (non-GAAP)</t>
+          <t xml:space="preserve">      total gross reserves</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
-        <v>11760</v>
-      </c>
-      <c r="C60" s="3" t="n">
-        <v>12173</v>
-      </c>
-      <c r="D60" s="3" t="n">
-        <v>14688</v>
-      </c>
-      <c r="E60" s="3" t="n">
-        <v>15213</v>
-      </c>
+        <v>109983</v>
+      </c>
+      <c r="C60" s="3" t="n"/>
+      <c r="D60" s="3" t="n"/>
+      <c r="E60" s="3" t="n"/>
       <c r="F60" s="3" t="n">
-        <v>16837</v>
+        <v>122473</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>17080</v>
+        <v>122911</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      total net reserves</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="n">
+        <v>97894</v>
+      </c>
+      <c r="C61" s="3" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n">
+        <v>110321</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>110974</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="inlineStr">
-        <is>
-          <t>⑥ CROSS-GATE — 2025 quarters vs FY2025 (Engine-FY column D)</t>
-        </is>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Total equity</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="n">
+        <v>13076</v>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>13010</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>15839</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>16915</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>17917</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>16891</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
+          <t>CHECK: A = L + E</t>
+        </is>
+      </c>
+      <c r="B63" s="4">
+        <f>IF(OR(B58+B62="",B56=""),"n/a",IF(ABS(B58+B62-B56)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="C63" s="4">
+        <f>IF(OR(C58+C62="",C56=""),"n/a",IF(ABS(C58+C62-C56)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="D63" s="4">
+        <f>IF(OR(D58+D62="",D56=""),"n/a",IF(ABS(D58+D62-D56)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="E63" s="4">
+        <f>IF(OR(E58+E62="",E56=""),"n/a",IF(ABS(E58+E62-E56)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="F63" s="4">
+        <f>IF(OR(F58+F62="",F56=""),"n/a",IF(ABS(F58+F62-F56)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="G63" s="4">
+        <f>IF(OR(G58+G62="",G56=""),"n/a",IF(ABS(G58+G62-G56)&lt;=2,"OK","FAIL"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted equity (non-GAAP)</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="n">
+        <v>11760</v>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>12173</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>14688</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>15213</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>16837</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>17080</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>⑥ CROSS-GATE — 2025 quarters vs FY2025 (Engine-FY column D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
           <t>CHECK: Σ(1Q25..4Q25) net income = FY2025</t>
         </is>
       </c>
-      <c r="B63" s="4">
+      <c r="B67" s="4">
         <f>IF(ABS(SUM(C13:F13)-'Engine-FY'!D48)&lt;=2,"OK","FAIL")</f>
         <v/>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>CHECK: Σ(1Q25..4Q25) DOE = FY2025</t>
         </is>
       </c>
-      <c r="B64" s="4">
+      <c r="B68" s="4">
         <f>IF(ABS(SUM(C10:F10)-'Engine-FY'!D62)&lt;=2,"OK","FAIL")</f>
         <v/>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>CHECK: Σ(1Q25..4Q25) gross annuity sales = FY2025</t>
         </is>
       </c>
-      <c r="B65" s="4">
-        <f>IF(ABS(SUM(C39:F39)-'Engine-FY'!D13)&lt;=2,"OK","FAIL")</f>
+      <c r="B69" s="4">
+        <f>IF(ABS(SUM(C43:F43)-'Engine-FY'!D13)&lt;=2,"OK","FAIL")</f>
         <v/>
       </c>
     </row>
@@ -3181,12 +3304,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>TOTAL FAILING CHECKS</t>
         </is>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="5">
         <f>B3+B4+B5+B6</f>
         <v/>
       </c>
@@ -3220,7 +3343,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF('Engine'!C21,"FAIL")+COUNTIF('Engine'!D21,"FAIL")+COUNTIF('Engine'!E21,"FAIL")+COUNTIF('Engine'!F21,"FAIL")+COUNTIF('Engine'!G21,"FAIL")+COUNTIF('Engine'!B34,"FAIL")+COUNTIF('Engine'!C34,"FAIL")+COUNTIF('Engine'!D34,"FAIL")+COUNTIF('Engine'!E34,"FAIL")+COUNTIF('Engine'!F34,"FAIL")+COUNTIF('Engine'!G34,"FAIL")+COUNTIF('Engine'!B38,"FAIL")+COUNTIF('Engine'!C38,"FAIL")+COUNTIF('Engine'!D38,"FAIL")+COUNTIF('Engine'!E38,"FAIL")+COUNTIF('Engine'!F38,"FAIL")+COUNTIF('Engine'!G38,"FAIL")+COUNTIF('Engine'!B40,"FAIL")+COUNTIF('Engine'!C40,"FAIL")+COUNTIF('Engine'!D40,"FAIL")+COUNTIF('Engine'!E40,"FAIL")+COUNTIF('Engine'!F40,"FAIL")+COUNTIF('Engine'!G40,"FAIL")+COUNTIF('Engine'!B59,"FAIL")+COUNTIF('Engine'!C59,"FAIL")+COUNTIF('Engine'!D59,"FAIL")+COUNTIF('Engine'!E59,"FAIL")+COUNTIF('Engine'!F59,"FAIL")+COUNTIF('Engine'!G59,"FAIL")</f>
+        <f>COUNTIF('Engine'!C21,"FAIL")+COUNTIF('Engine'!D21,"FAIL")+COUNTIF('Engine'!E21,"FAIL")+COUNTIF('Engine'!F21,"FAIL")+COUNTIF('Engine'!G21,"FAIL")+COUNTIF('Engine'!B27,"FAIL")+COUNTIF('Engine'!C27,"FAIL")+COUNTIF('Engine'!D27,"FAIL")+COUNTIF('Engine'!E27,"FAIL")+COUNTIF('Engine'!F27,"FAIL")+COUNTIF('Engine'!G27,"FAIL")+COUNTIF('Engine'!B38,"FAIL")+COUNTIF('Engine'!C38,"FAIL")+COUNTIF('Engine'!D38,"FAIL")+COUNTIF('Engine'!E38,"FAIL")+COUNTIF('Engine'!F38,"FAIL")+COUNTIF('Engine'!G38,"FAIL")+COUNTIF('Engine'!B42,"FAIL")+COUNTIF('Engine'!C42,"FAIL")+COUNTIF('Engine'!D42,"FAIL")+COUNTIF('Engine'!E42,"FAIL")+COUNTIF('Engine'!F42,"FAIL")+COUNTIF('Engine'!G42,"FAIL")+COUNTIF('Engine'!B44,"FAIL")+COUNTIF('Engine'!C44,"FAIL")+COUNTIF('Engine'!D44,"FAIL")+COUNTIF('Engine'!E44,"FAIL")+COUNTIF('Engine'!F44,"FAIL")+COUNTIF('Engine'!G44,"FAIL")</f>
         <v/>
       </c>
     </row>
@@ -3231,14 +3354,14 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF('Engine'!B63,"FAIL")+COUNTIF('Engine'!B64,"FAIL")+COUNTIF('Engine'!B65,"FAIL")</f>
+        <f>COUNTIF('Engine'!B63,"FAIL")+COUNTIF('Engine'!C63,"FAIL")+COUNTIF('Engine'!D63,"FAIL")+COUNTIF('Engine'!E63,"FAIL")+COUNTIF('Engine'!F63,"FAIL")+COUNTIF('Engine'!G63,"FAIL")+COUNTIF('Engine'!B67,"FAIL")+COUNTIF('Engine'!B68,"FAIL")+COUNTIF('Engine'!B69,"FAIL")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>87 check cells tracked. BNT engine.</t>
+          <t>93 check cells tracked. BNT engine.</t>
         </is>
       </c>
     </row>

</xml_diff>